<commit_message>
techs and vendors cards
</commit_message>
<xml_diff>
--- a/docs/ONC Hydrophones Specs.xlsx
+++ b/docs/ONC Hydrophones Specs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ebeaudin/Desktop/Hydrophones/hydrophone-handbook/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33735C0-1684-3B47-9BBF-2EDED1335BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714899F6-7A20-E545-8B46-4E354AECDEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -772,7 +772,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="32.1640625" customWidth="1"/>
@@ -885,24 +885,50 @@
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
     </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+    </row>
     <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
@@ -913,22 +939,14 @@
     </row>
     <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>41</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
@@ -939,14 +957,22 @@
     </row>
     <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>46</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
@@ -957,22 +983,22 @@
     </row>
     <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>46</v>
+        <v>51</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -983,22 +1009,20 @@
     </row>
     <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7">
+        <v>-173</v>
+      </c>
+      <c r="F9" s="8">
+        <v>-169</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
@@ -1009,20 +1033,22 @@
     </row>
     <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7">
-        <v>-173</v>
-      </c>
-      <c r="F10" s="8">
-        <v>-169</v>
+        <v>58</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
@@ -1033,22 +1059,22 @@
     </row>
     <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>60</v>
+        <v>65</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -1059,22 +1085,22 @@
     </row>
     <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>66</v>
+        <v>69</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -1085,22 +1111,18 @@
     </row>
     <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="15">
+        <v>0.5</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
@@ -1111,18 +1133,22 @@
     </row>
     <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="14">
-        <v>0.5</v>
-      </c>
-      <c r="F14" s="15">
-        <v>0.5</v>
+        <v>72</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1131,24 +1157,24 @@
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
     </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="F15" s="8" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -1157,24 +1183,24 @@
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" spans="1:12" ht="51" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>45</v>
+        <v>78</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -1183,24 +1209,20 @@
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
     </row>
-    <row r="17" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
@@ -1211,18 +1233,22 @@
     </row>
     <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
+        <v>83</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>84</v>
+      </c>
       <c r="D18" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -1233,22 +1259,22 @@
     </row>
     <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
@@ -1257,45 +1283,47 @@
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
     </row>
-    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-    </row>
-    <row r="36" spans="1:26" ht="18" x14ac:dyDescent="0.2">
-      <c r="A36" s="19"/>
-      <c r="C36" s="16"/>
+    <row r="35" spans="1:26" ht="18" x14ac:dyDescent="0.2">
+      <c r="A35" s="19"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+    </row>
+    <row r="36" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-    </row>
-    <row r="37" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D37" s="16"/>
+    </row>
+    <row r="37" spans="1:26" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="20"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18"/>
+      <c r="O37" s="18"/>
+      <c r="P37" s="18"/>
+      <c r="Q37" s="18"/>
+      <c r="R37" s="18"/>
+      <c r="S37" s="18"/>
+      <c r="T37" s="18"/>
+      <c r="U37" s="18"/>
+      <c r="V37" s="18"/>
+      <c r="W37" s="18"/>
+      <c r="X37" s="18"/>
+      <c r="Y37" s="18"/>
+      <c r="Z37" s="18"/>
     </row>
     <row r="38" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="20"/>
-      <c r="B38" s="21"/>
+      <c r="B38" s="22"/>
       <c r="C38" s="21"/>
       <c r="D38" s="22"/>
       <c r="E38" s="22"/>
@@ -1305,25 +1333,11 @@
       <c r="I38" s="17"/>
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="18"/>
-      <c r="N38" s="18"/>
-      <c r="O38" s="18"/>
-      <c r="P38" s="18"/>
-      <c r="Q38" s="18"/>
-      <c r="R38" s="18"/>
-      <c r="S38" s="18"/>
-      <c r="T38" s="18"/>
-      <c r="U38" s="18"/>
-      <c r="V38" s="18"/>
-      <c r="W38" s="18"/>
-      <c r="X38" s="18"/>
-      <c r="Y38" s="18"/>
-      <c r="Z38" s="18"/>
+      <c r="L38" s="8"/>
     </row>
     <row r="39" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="20"/>
-      <c r="B39" s="22"/>
+      <c r="B39" s="21"/>
       <c r="C39" s="21"/>
       <c r="D39" s="22"/>
       <c r="E39" s="22"/>
@@ -1333,43 +1347,43 @@
       <c r="I39" s="17"/>
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
-      <c r="L39" s="8"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="18"/>
+      <c r="Q39" s="18"/>
+      <c r="R39" s="18"/>
+      <c r="S39" s="18"/>
+      <c r="T39" s="18"/>
+      <c r="U39" s="18"/>
+      <c r="V39" s="18"/>
+      <c r="W39" s="18"/>
+      <c r="X39" s="18"/>
+      <c r="Y39" s="18"/>
+      <c r="Z39" s="18"/>
     </row>
     <row r="40" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="20"/>
-      <c r="B40" s="21"/>
+      <c r="B40" s="22"/>
       <c r="C40" s="21"/>
       <c r="D40" s="22"/>
       <c r="E40" s="22"/>
       <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="18"/>
-      <c r="N40" s="18"/>
-      <c r="O40" s="18"/>
-      <c r="P40" s="18"/>
-      <c r="Q40" s="18"/>
-      <c r="R40" s="18"/>
-      <c r="S40" s="18"/>
-      <c r="T40" s="18"/>
-      <c r="U40" s="18"/>
-      <c r="V40" s="18"/>
-      <c r="W40" s="18"/>
-      <c r="X40" s="18"/>
-      <c r="Y40" s="18"/>
-      <c r="Z40" s="18"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
     </row>
     <row r="41" spans="1:26" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" s="20"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="17"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="8"/>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
       <c r="I41" s="8"/>
@@ -1378,60 +1392,49 @@
       <c r="L41" s="8"/>
     </row>
     <row r="42" spans="1:26" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="4"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="8"/>
-      <c r="K42" s="8"/>
-      <c r="L42" s="8"/>
+      <c r="A42" s="20"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="17"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="17"/>
+      <c r="L42" s="17"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
+      <c r="O42" s="18"/>
+      <c r="P42" s="18"/>
+      <c r="Q42" s="18"/>
+      <c r="R42" s="18"/>
+      <c r="S42" s="18"/>
+      <c r="T42" s="18"/>
+      <c r="U42" s="18"/>
+      <c r="V42" s="18"/>
+      <c r="W42" s="18"/>
+      <c r="X42" s="18"/>
+      <c r="Y42" s="18"/>
+      <c r="Z42" s="18"/>
     </row>
     <row r="43" spans="1:26" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="20"/>
-      <c r="B43" s="21"/>
-      <c r="C43" s="21"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="18"/>
-      <c r="N43" s="18"/>
-      <c r="O43" s="18"/>
-      <c r="P43" s="18"/>
-      <c r="Q43" s="18"/>
-      <c r="R43" s="18"/>
-      <c r="S43" s="18"/>
-      <c r="T43" s="18"/>
-      <c r="U43" s="18"/>
-      <c r="V43" s="18"/>
-      <c r="W43" s="18"/>
-      <c r="X43" s="18"/>
-      <c r="Y43" s="18"/>
-      <c r="Z43" s="18"/>
-    </row>
-    <row r="44" spans="1:26" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="4"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="8"/>
+    </row>
+    <row r="44" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D44" s="16"/>
     </row>
     <row r="45" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D45" s="16"/>
@@ -1481,7 +1484,7 @@
     <row r="60" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D60" s="16"/>
     </row>
-    <row r="61" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="4:4" ht="13" x14ac:dyDescent="0.15">
       <c r="D61" s="16"/>
     </row>
     <row r="62" spans="4:4" ht="13" x14ac:dyDescent="0.15">
@@ -4294,9 +4297,6 @@
     </row>
     <row r="998" spans="4:4" ht="13" x14ac:dyDescent="0.15">
       <c r="D998" s="16"/>
-    </row>
-    <row r="999" spans="4:4" ht="13" x14ac:dyDescent="0.15">
-      <c r="D999" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
scattered how hydrophones work info
</commit_message>
<xml_diff>
--- a/docs/ONC Hydrophones Specs.xlsx
+++ b/docs/ONC Hydrophones Specs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ebeaudin/Desktop/Hydrophones/hydrophone-handbook/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714899F6-7A20-E545-8B46-4E354AECDEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{029699B6-38B1-F545-9ECA-F1F353BAC254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -266,19 +266,10 @@
     <t>Frequency Range</t>
   </si>
   <si>
-    <t>1 Hz - 200 KHz</t>
-  </si>
-  <si>
     <t>10 kHz - 200 kHz</t>
   </si>
   <si>
-    <t>1 - 1600 Hz (infrasound)</t>
-  </si>
-  <si>
     <t>10 Hz - 200 kHz (effective up to 128 kHz)</t>
-  </si>
-  <si>
-    <t>10 Hz - 10 kHz</t>
   </si>
   <si>
     <t>Operating Temperatures</t>
@@ -348,6 +339,15 @@
   </si>
   <si>
     <t>SubConn MCBH8-M</t>
+  </si>
+  <si>
+    <t>10 Hz - 12 kHz</t>
+  </si>
+  <si>
+    <t>0.1 - 1600 Hz (infrasound)</t>
+  </si>
+  <si>
+    <t>1 Hz - 200 kHz</t>
   </si>
 </sst>
 </file>
@@ -1062,19 +1062,19 @@
         <v>61</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>65</v>
-      </c>
       <c r="F11" s="12" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -1085,22 +1085,22 @@
     </row>
     <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>70</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="13"/>
@@ -1133,7 +1133,7 @@
     </row>
     <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>45</v>
@@ -1142,13 +1142,13 @@
         <v>45</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1159,13 +1159,13 @@
     </row>
     <row r="15" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>45</v>
@@ -1185,22 +1185,22 @@
     </row>
     <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>80</v>
-      </c>
       <c r="F16" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -1211,18 +1211,18 @@
     </row>
     <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
@@ -1233,22 +1233,22 @@
     </row>
     <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -1259,22 +1259,22 @@
     </row>
     <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>88</v>
-      </c>
       <c r="E19" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
@@ -4308,7 +4308,7 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>25</v>
       </c>

</xml_diff>